<commit_message>
Simplify step UI to image+text and use .env DATABASE_URL
- Steps now hold only an image + text description; remove decision
  question, normal/next labels, result text, next_step_order, caution,
  and step_title from model, schema, router, DB, and import pipeline
- Viewer offers two actions: 정상/조치 완료 (done) and 추가 정보 필요
  (auto-advance; escalate message on last step)
- New-guide flow: type-selection modal routes to /guides/new?type=; form
  labels and page titles switch by ALARM/INTERLOCK
- Import template reduced to step{1..5}_description (step1 required)
- Read DATABASE_URL from backend/.env via python-dotenv; never hardcode;
  create_all only when AUTO_CREATE_TABLES=true (no drops/seed); schema.sql
  is reference-only, non-destructive, targets cmpbeol DB

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/alarm_sample.xlsx
+++ b/samples/alarm_sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,77 +461,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>step1_title</t>
+          <t>step1_description</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>step1_description</t>
+          <t>step2_description</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>step1_question</t>
+          <t>step3_description</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>step1_normal_result</t>
+          <t>step4_description</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>step1_caution</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>step2_title</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>step2_description</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>step2_question</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>step2_normal_result</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>step2_caution</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>step3_title</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>step3_description</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>step3_question</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>step3_normal_result</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>step3_caution</t>
+          <t>step5_description</t>
         </is>
       </c>
     </row>
@@ -568,75 +518,21 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>슬러리 공급 압력 확인</t>
+          <t>슬러리 공급 라인 압력 게이지를 확인한다. (분출 주의 보호구 착용)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>슬러리 공급 라인 압력 게이지를 확인한다</t>
+          <t>슬러리 필터 차압 게이지를 확인한다</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>공급 압력이 정상 범위인가요?</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>압력 정상. 유량계 표시값을 확인하세요.</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>슬러리 분출 주의 보호구 착용</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>필터 차압 확인</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>슬러리 필터 차압 게이지를 확인한다</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>필터 차압이 정상 범위인가요?</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>필터 정상. 펌프 동작을 확인하세요.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>펌프 재기동</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>다이어프램 펌프를 재기동한다</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>유량이 회복되었나요?</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>유량 정상 회복. 조치 완료.</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>해결 안되면 담당자 문의</t>
-        </is>
-      </c>
+          <t>다이어프램 펌프를 재기동하고 유량 회복을 확인한다</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -671,142 +567,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>헤드 회전 이상음 확인</t>
+          <t>설비 안전 정지 후 헤드 회전부를 육안 점검한다. (과열 상태 재기동 금지)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>설비 안전 정지 후 헤드 회전부를 육안 점검한다</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>기계적 걸림/이상음이 없나요?</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>기계부 정상. 다운포스 설정을 확인하세요.</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>과열 상태 재기동 금지</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>다운포스 재설정</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
           <t>다운포스를 정상 범위로 재설정 후 무부하 시운전한다</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>시운전이 정상인가요?</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>정상 확인. 조치 완료.</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>INTERLOCK</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>LK</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DOOR_OPEN_INT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Door Open Interlock</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>CMP</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>도어 개방 인터락 발생 시 조치 가이드</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Door Sensor 상태 확인</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Door sensor LED 상태를 확인한다</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Sensor LED가 정상 점등 상태인가요?</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>정상으로 판단되어 추가 조치가 필요하지 않습니다.</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Door 개방 시 안전 유의</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Door 폐쇄 및 리셋</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>내부 잔류 확인 후 도어를 완전히 닫고 리셋한다</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>도어 스위치 신호가 정상인가요?</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>정상 확인. 조치 완료.</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>내부 안전 확인 필수</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>